<commit_message>
SI 4: correct amplicon positions and lengths, fix one-base deletion in Amphipoda amplicon
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/supporting information/supporting information 4.xlsx
+++ b/supporting information/supporting information 4.xlsx
@@ -512,17 +512,17 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="G2" t="n">
         <v>365</v>
       </c>
       <c r="H2" t="n">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>GGCTTGTAGAAAGGGGAGTCGGTACAGGTTGGACTGTCTACCCCCCGCTAGCGGGGGCAGTAGCCCACAGAGGGGGTGCGGTAGACTTGGCTATTTTTCTCTACACCTGGCTGGTGCTTCCTCTATCTTAGGCGC</t>
+          <t>GGCTTGTAGAAAGGGGAGTCGGTACAGGTTGGACTGTCTACCCCCCGCTAGCGGGGGCAGTAGCCCACAGAGGGGGTGCGGTAGACTTGGCTATTTTTTCTCTACACCTGGCTGGTGCTTCCTCTATCTTAGGCGC</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G3" t="n">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="H3" t="n">
         <v>104</v>
@@ -625,7 +625,7 @@
         <v>199</v>
       </c>
       <c r="G4" t="n">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="H4" t="n">
         <v>147</v>
@@ -732,10 +732,10 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G6" t="n">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="H6" t="n">
         <v>163</v>

</xml_diff>